<commit_message>
Add Signature Form Before Export
</commit_message>
<xml_diff>
--- a/public/templates/Kontrak_Manajemen.xlsx
+++ b/public/templates/Kontrak_Manajemen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghifa\Documents\admin-dashboard\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C63FA22-905D-422C-B480-B56A4B6D1F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{198351AE-D80B-479C-8DA7-668969751F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BFAE523-3C32-487F-867A-BFB50E6068E4}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>SASARAN STRATEGIS</t>
   </si>
@@ -81,13 +81,7 @@
     <t>S (Support)        :     Pendukung</t>
   </si>
   <si>
-    <t>IIP ARIEF BUDIMAN</t>
-  </si>
-  <si>
     <t>Direktur Utama</t>
-  </si>
-  <si>
-    <t>GESRANG TARIGAN</t>
   </si>
   <si>
     <t>Plt. Direktur Keungan &amp; SDM</t>
@@ -233,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -278,6 +272,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -909,63 +906,69 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>13</v>
       </c>
       <c r="B34" s="15"/>
       <c r="C34" s="15"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
         <v>12</v>
       </c>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
         <v>14</v>
       </c>
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B43" s="8" t="s">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B43" s="8"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="8"/>
+      <c r="I43" s="8"/>
+      <c r="J43" s="8"/>
+      <c r="K43" s="8"/>
+      <c r="L43" s="8"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B44" s="9" t="s">
         <v>15</v>
-      </c>
-      <c r="C43" s="9"/>
-      <c r="D43" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="I43" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="J43" s="9"/>
-      <c r="K43" s="9"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B44" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E44" s="9"/>
       <c r="F44" s="9"/>
-      <c r="G44" s="7"/>
-      <c r="H44" s="7"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
       <c r="I44" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J44" s="9"/>
       <c r="K44" s="9"/>
+      <c r="L44" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
+    <mergeCell ref="D38:H38"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A36:C36"/>
@@ -981,10 +984,10 @@
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="B44:C44"/>
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:L43"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="I44:L44"/>
+    <mergeCell ref="D44:H44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>